<commit_message>
fix: require explicit wave numeric data
</commit_message>
<xml_diff>
--- a/Excel/waves#波次.xlsx
+++ b/Excel/waves#波次.xlsx
@@ -1223,9 +1223,8 @@
       <c r="A4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="1">
-        <f>D4/E4</f>
-        <v/>
+      <c r="B4" s="1" t="n">
+        <v>64</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>1</v>
@@ -1256,9 +1255,8 @@
       <c r="A5" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="1">
-        <f>D5/E5</f>
-        <v/>
+      <c r="B5" s="1" t="n">
+        <v>64</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>1</v>
@@ -1289,9 +1287,8 @@
       <c r="A6" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="1">
-        <f>D6/E6</f>
-        <v/>
+      <c r="B6" s="1" t="n">
+        <v>64</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>1</v>
@@ -1322,9 +1319,8 @@
       <c r="A7" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="1">
-        <f>D7/E7</f>
-        <v/>
+      <c r="B7" s="1" t="n">
+        <v>64</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>1</v>
@@ -1355,9 +1351,8 @@
       <c r="A8" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="1">
-        <f>D8/E8</f>
-        <v/>
+      <c r="B8" s="1" t="n">
+        <v>64</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>1</v>
@@ -1388,9 +1383,8 @@
       <c r="A9" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="1">
-        <f>D9/E9</f>
-        <v/>
+      <c r="B9" s="1" t="n">
+        <v>80</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>1</v>
@@ -1421,9 +1415,8 @@
       <c r="A10" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="1">
-        <f>D10/E10</f>
-        <v/>
+      <c r="B10" s="1" t="n">
+        <v>80</v>
       </c>
       <c r="C10" s="1" t="n">
         <v>1</v>
@@ -1454,9 +1447,8 @@
       <c r="A11" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="1">
-        <f>D11/E11</f>
-        <v/>
+      <c r="B11" s="1" t="n">
+        <v>80</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>1</v>
@@ -1487,9 +1479,8 @@
       <c r="A12" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="1">
-        <f>D12/E12</f>
-        <v/>
+      <c r="B12" s="1" t="n">
+        <v>80</v>
       </c>
       <c r="C12" s="1" t="n">
         <v>1</v>
@@ -1520,9 +1511,8 @@
       <c r="A13" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="1">
-        <f>D13/E13</f>
-        <v/>
+      <c r="B13" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1535,6 +1525,13 @@
       </c>
       <c r="F13" s="1" t="n">
         <v>1003010</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
       </c>
       <c r="J13" s="1" t="n">
         <v>2</v>
@@ -1544,9 +1541,8 @@
       <c r="A14" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="1">
-        <f>D14/E14</f>
-        <v/>
+      <c r="B14" s="1" t="n">
+        <v>100</v>
       </c>
       <c r="C14" s="1" t="n">
         <v>1</v>
@@ -1577,9 +1573,8 @@
       <c r="A15" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="1">
-        <f>D15/E15</f>
-        <v/>
+      <c r="B15" s="1" t="n">
+        <v>100</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>1</v>
@@ -1610,9 +1605,8 @@
       <c r="A16" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="1">
-        <f>D16/E16</f>
-        <v/>
+      <c r="B16" s="1" t="n">
+        <v>100</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>1</v>
@@ -1643,9 +1637,8 @@
       <c r="A17" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="1">
-        <f>D17/E17</f>
-        <v/>
+      <c r="B17" s="1" t="n">
+        <v>100</v>
       </c>
       <c r="C17" s="1" t="n">
         <v>1</v>
@@ -1676,9 +1669,8 @@
       <c r="A18" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="1">
-        <f>D18/E18</f>
-        <v/>
+      <c r="B18" s="1" t="n">
+        <v>100</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
@@ -1709,9 +1701,8 @@
       <c r="A19" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="1">
-        <f>D19/E19</f>
-        <v/>
+      <c r="B19" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
@@ -1742,9 +1733,8 @@
       <c r="A20" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="1">
-        <f>D20/E20</f>
-        <v/>
+      <c r="B20" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C20" s="1" t="n">
         <v>1</v>
@@ -1775,9 +1765,8 @@
       <c r="A21" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="1">
-        <f>D21/E21</f>
-        <v/>
+      <c r="B21" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C21" s="1" t="n">
         <v>1</v>
@@ -1840,9 +1829,8 @@
       <c r="A23" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="1">
-        <f>D23/E23</f>
-        <v/>
+      <c r="B23" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="C23" s="1" t="n">
         <v>1</v>
@@ -1855,6 +1843,13 @@
       </c>
       <c r="F23" s="1" t="n">
         <v>1003020</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
       </c>
       <c r="J23" s="1" t="n">
         <v>2</v>
@@ -1864,9 +1859,8 @@
       <c r="A24" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="1">
-        <f>D24/E24</f>
-        <v/>
+      <c r="B24" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C24" s="1" t="n">
         <v>1</v>
@@ -1897,9 +1891,8 @@
       <c r="A25" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="1">
-        <f>D25/E25</f>
-        <v/>
+      <c r="B25" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C25" s="1" t="n">
         <v>1</v>
@@ -1930,9 +1923,8 @@
       <c r="A26" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="1">
-        <f>D26/E26</f>
-        <v/>
+      <c r="B26" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C26" s="1" t="n">
         <v>1</v>
@@ -1963,9 +1955,8 @@
       <c r="A27" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="1">
-        <f>D27/E27</f>
-        <v/>
+      <c r="B27" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C27" s="1" t="n">
         <v>1</v>
@@ -1996,9 +1987,8 @@
       <c r="A28" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="1">
-        <f>D28/E28</f>
-        <v/>
+      <c r="B28" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C28" s="1" t="n">
         <v>1</v>
@@ -2029,9 +2019,8 @@
       <c r="A29" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="1">
-        <f>D29/E29</f>
-        <v/>
+      <c r="B29" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C29" s="1" t="n">
         <v>1</v>
@@ -2062,9 +2051,8 @@
       <c r="A30" s="1" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="1">
-        <f>D30/E30</f>
-        <v/>
+      <c r="B30" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C30" s="1" t="n">
         <v>1</v>
@@ -2095,9 +2083,8 @@
       <c r="A31" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="1">
-        <f>D31/E31</f>
-        <v/>
+      <c r="B31" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C31" s="1" t="n">
         <v>1</v>
@@ -2128,9 +2115,8 @@
       <c r="A32" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="1">
-        <f>D32/E32</f>
-        <v/>
+      <c r="B32" s="1" t="n">
+        <v>160</v>
       </c>
       <c r="C32" s="1" t="n">
         <v>1</v>
@@ -2161,9 +2147,8 @@
       <c r="A33" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="1">
-        <f>D33/E33</f>
-        <v/>
+      <c r="B33" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="C33" s="1" t="n">
         <v>1</v>
@@ -2176,6 +2161,13 @@
       </c>
       <c r="F33" s="1" t="n">
         <v>1003030</v>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
       </c>
       <c r="J33" s="1" t="n">
         <v>2</v>

</xml_diff>